<commit_message>
feat: Datos actualizados con EAN
</commit_message>
<xml_diff>
--- a/frontend/public/reports/StockPulse_REPRESENTADAS.xlsx
+++ b/frontend/public/reports/StockPulse_REPRESENTADAS.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="791" uniqueCount="517">
   <si>
     <t>#</t>
   </si>
@@ -37,252 +37,366 @@
     <t>85005</t>
   </si>
   <si>
+    <t>7754807850056</t>
+  </si>
+  <si>
+    <t>LIGAS N° 18 - 80 MM X 2 MM X 1 LBS - NATURAL - ALLEANZA</t>
+  </si>
+  <si>
+    <t>✓ OK</t>
+  </si>
+  <si>
+    <t>85007</t>
+  </si>
+  <si>
+    <t>7754807850063</t>
+  </si>
+  <si>
+    <t>LIGAS N° 18 - 80 MM X 2 MM X 1/4 LBS - NATURAL - ALLEANZA</t>
+  </si>
+  <si>
+    <t>85768</t>
+  </si>
+  <si>
+    <t>7754807857680</t>
+  </si>
+  <si>
+    <t>LIGAS N° 18 - 80 MM X 2 MM X 1/4 LBS - VERDE - ALLEANZA</t>
+  </si>
+  <si>
+    <t>85008</t>
+  </si>
+  <si>
+    <t>7754807850087</t>
+  </si>
+  <si>
+    <t>LIGAS N° 78 - 140 MM X 10 MM X 1 LBS - NATURAL - ALLEANZA</t>
+  </si>
+  <si>
+    <t>85801</t>
+  </si>
+  <si>
+    <t>7754807857024</t>
+  </si>
+  <si>
+    <t>ALFILER ALLEANZA 35 MM CAJA X 50 GR</t>
+  </si>
+  <si>
+    <t>85163</t>
+  </si>
+  <si>
+    <t>091511400595</t>
+  </si>
+  <si>
+    <t>CUCHILLA ARTE AK-1/5B</t>
+  </si>
+  <si>
+    <t>85164</t>
+  </si>
+  <si>
+    <t>091511400670</t>
+  </si>
+  <si>
+    <t>CUCHILLA ARTE AK-4</t>
+  </si>
+  <si>
+    <t>85770</t>
+  </si>
+  <si>
+    <t>091511220292</t>
+  </si>
+  <si>
+    <t>CUCHILLA ARTE AK-5 + KB-5/30B</t>
+  </si>
+  <si>
+    <t>85868</t>
+  </si>
+  <si>
+    <t>4901165202925</t>
+  </si>
+  <si>
+    <t>CUCHILLLA ARTE AK-5 PINK</t>
+  </si>
+  <si>
+    <t>85871</t>
+  </si>
+  <si>
+    <t>CUCHILLLA DE ARTE AK-5/5B</t>
+  </si>
+  <si>
+    <t>✗ AGOTADO</t>
+  </si>
+  <si>
+    <t>85166</t>
+  </si>
+  <si>
+    <t>091511400441</t>
+  </si>
+  <si>
+    <t>CUCHILLA ARTE MC-45/2B</t>
+  </si>
+  <si>
+    <t>85172</t>
+  </si>
+  <si>
+    <t>091511400144</t>
+  </si>
+  <si>
+    <t>CUCHILLA COMPAS CMP-1</t>
+  </si>
+  <si>
+    <t>85171</t>
+  </si>
+  <si>
+    <t>091511400786</t>
+  </si>
+  <si>
+    <t>CUCHILLA COMPAS CMP-1 DX</t>
+  </si>
+  <si>
+    <t>85174</t>
+  </si>
+  <si>
+    <t>091511100334</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY BN-AL</t>
+  </si>
+  <si>
+    <t>85175</t>
+  </si>
+  <si>
+    <t>091511100327</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY BN-L</t>
+  </si>
+  <si>
+    <t>85179</t>
+  </si>
+  <si>
+    <t>091511200515</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY DL-1</t>
+  </si>
+  <si>
+    <t>85180</t>
+  </si>
+  <si>
+    <t>091511200300</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY EXL</t>
+  </si>
+  <si>
+    <t>85183</t>
+  </si>
+  <si>
+    <t>091511200195</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY L-1</t>
+  </si>
+  <si>
+    <t>85889</t>
+  </si>
+  <si>
+    <t>091511900019</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY L-1 GREEN</t>
+  </si>
+  <si>
+    <t>85185</t>
+  </si>
+  <si>
+    <t>091511200102</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY L-2</t>
+  </si>
+  <si>
+    <t>85187</t>
+  </si>
+  <si>
+    <t>091511200461</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY L-5</t>
+  </si>
+  <si>
+    <t>85623</t>
+  </si>
+  <si>
+    <t>091511200447</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY L-5 AL</t>
+  </si>
+  <si>
+    <t>⚠ BAJO</t>
+  </si>
+  <si>
+    <t>85823</t>
+  </si>
+  <si>
+    <t>091511220469</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY L-7</t>
+  </si>
+  <si>
+    <t>85824</t>
+  </si>
+  <si>
+    <t>091511220315</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY L-7 AL</t>
+  </si>
+  <si>
+    <t>85190</t>
+  </si>
+  <si>
+    <t>091511200270</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY ML</t>
+  </si>
+  <si>
+    <t>85192</t>
+  </si>
+  <si>
+    <t>091511200157</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY OL</t>
+  </si>
+  <si>
+    <t>85194</t>
+  </si>
+  <si>
+    <t>091511200126</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY SL-1</t>
+  </si>
+  <si>
+    <t>85887</t>
+  </si>
+  <si>
+    <t>091511200478</t>
+  </si>
+  <si>
+    <t>CUCHILLA HEAVY DUTY XH-1</t>
+  </si>
+  <si>
+    <t>85196</t>
+  </si>
+  <si>
+    <t>091511400946</t>
+  </si>
+  <si>
+    <t>CUCHILLA PLASTIC CUTTER PC-L</t>
+  </si>
+  <si>
+    <t>85173</t>
+  </si>
+  <si>
+    <t>091511900217</t>
+  </si>
+  <si>
+    <t>CUCHILLA SEGURIDAD SK-10</t>
+  </si>
+  <si>
+    <t>85167</t>
+  </si>
+  <si>
+    <t>091511400625</t>
+  </si>
+  <si>
+    <t>CUCHILLA SEGURIDAD SK-4</t>
+  </si>
+  <si>
+    <t>85863</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>LIGAS N° 18 - 80 MM X 2 MM X 1 LBS - NATURAL - ALLEANZA</t>
-  </si>
-  <si>
-    <t>✓ OK</t>
-  </si>
-  <si>
-    <t>85007</t>
-  </si>
-  <si>
-    <t>LIGAS N° 18 - 80 MM X 2 MM X 1/4 LBS - NATURAL - ALLEANZA</t>
-  </si>
-  <si>
-    <t>85768</t>
-  </si>
-  <si>
-    <t>LIGAS N° 18 - 80 MM X 2 MM X 1/4 LBS - VERDE - ALLEANZA</t>
-  </si>
-  <si>
-    <t>85008</t>
-  </si>
-  <si>
-    <t>LIGAS N° 78 - 140 MM X 10 MM X 1 LBS - NATURAL - ALLEANZA</t>
-  </si>
-  <si>
-    <t>85801</t>
-  </si>
-  <si>
-    <t>ALFILER ALLEANZA 35 MM CAJA X 50 GR</t>
-  </si>
-  <si>
-    <t>85163</t>
-  </si>
-  <si>
-    <t>CUCHILLA ARTE AK-1/5B</t>
-  </si>
-  <si>
-    <t>85164</t>
-  </si>
-  <si>
-    <t>CUCHILLA ARTE AK-4</t>
-  </si>
-  <si>
-    <t>85770</t>
-  </si>
-  <si>
-    <t>CUCHILLA ARTE AK-5 + KB-5/30B</t>
-  </si>
-  <si>
-    <t>85868</t>
-  </si>
-  <si>
-    <t>CUCHILLLA ARTE AK-5 PINK</t>
-  </si>
-  <si>
-    <t>85871</t>
-  </si>
-  <si>
-    <t>CUCHILLLA DE ARTE AK-5/5B</t>
-  </si>
-  <si>
-    <t>✗ AGOTADO</t>
-  </si>
-  <si>
-    <t>85166</t>
-  </si>
-  <si>
-    <t>CUCHILLA ARTE MC-45/2B</t>
-  </si>
-  <si>
-    <t>85172</t>
-  </si>
-  <si>
-    <t>CUCHILLA COMPAS CMP-1</t>
-  </si>
-  <si>
-    <t>85171</t>
-  </si>
-  <si>
-    <t>CUCHILLA COMPAS CMP-1 DX</t>
-  </si>
-  <si>
-    <t>85174</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY BN-AL</t>
-  </si>
-  <si>
-    <t>85175</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY BN-L</t>
-  </si>
-  <si>
-    <t>85179</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY DL-1</t>
-  </si>
-  <si>
-    <t>85180</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY EXL</t>
-  </si>
-  <si>
-    <t>85183</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY L-1</t>
-  </si>
-  <si>
-    <t>85889</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY L-1 GREEN</t>
-  </si>
-  <si>
-    <t>85185</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY L-2</t>
-  </si>
-  <si>
-    <t>85187</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY L-5</t>
-  </si>
-  <si>
-    <t>85623</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY L-5 AL</t>
-  </si>
-  <si>
-    <t>⚠ BAJO</t>
-  </si>
-  <si>
-    <t>85823</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY L-7</t>
-  </si>
-  <si>
-    <t>85824</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY L-7 AL</t>
-  </si>
-  <si>
-    <t>85190</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY ML</t>
-  </si>
-  <si>
-    <t>85192</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY OL</t>
-  </si>
-  <si>
-    <t>85194</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY SL-1</t>
-  </si>
-  <si>
-    <t>85887</t>
-  </si>
-  <si>
-    <t>CUCHILLA HEAVY DUTY XH-1</t>
-  </si>
-  <si>
-    <t>85196</t>
-  </si>
-  <si>
-    <t>CUCHILLA PLASTIC CUTTER PC-L</t>
-  </si>
-  <si>
-    <t>85173</t>
-  </si>
-  <si>
-    <t>CUCHILLA SEGURIDAD SK-10</t>
-  </si>
-  <si>
-    <t>85167</t>
-  </si>
-  <si>
-    <t>CUCHILLA SEGURIDAD SK-4</t>
-  </si>
-  <si>
-    <t>85863</t>
-  </si>
-  <si>
     <t>CUCHILLA SEGURIDAD SK-4/24</t>
   </si>
   <si>
     <t>85168</t>
   </si>
   <si>
+    <t>091511400908</t>
+  </si>
+  <si>
     <t>CUCHILLA SEGURIDAD SK-9</t>
   </si>
   <si>
     <t>85861</t>
   </si>
   <si>
+    <t>091511610710</t>
+  </si>
+  <si>
     <t>CUCHILLA SEGURIDAD SK-9/32</t>
   </si>
   <si>
     <t>85870</t>
   </si>
   <si>
+    <t>091511230383</t>
+  </si>
+  <si>
     <t>CUCHILLA SEGURIDAD SK-16</t>
   </si>
   <si>
     <t>85206</t>
   </si>
   <si>
+    <t>091511400181</t>
+  </si>
+  <si>
     <t>CUCHILLA STANDARD 180 BLACK</t>
   </si>
   <si>
     <t>85207</t>
   </si>
   <si>
+    <t>091511100136</t>
+  </si>
+  <si>
     <t>CUCHILLA STANDARD 300</t>
   </si>
   <si>
     <t>85205</t>
   </si>
   <si>
+    <t>091511610796</t>
+  </si>
+  <si>
     <t>CUCHILLA STANDARD A-1</t>
   </si>
   <si>
     <t>85208</t>
   </si>
   <si>
+    <t>091511100129</t>
+  </si>
+  <si>
     <t>CUCHILLA STANDARD A-3</t>
   </si>
   <si>
     <t>85209</t>
   </si>
   <si>
+    <t>091511100471</t>
+  </si>
+  <si>
     <t>CUCHILLA STANDARD A-5</t>
   </si>
   <si>
@@ -295,30 +409,45 @@
     <t>85890</t>
   </si>
   <si>
+    <t>091511900026</t>
+  </si>
+  <si>
     <t>CUCHILLA STANDARD ES-1 GREEN</t>
   </si>
   <si>
     <t>85212</t>
   </si>
   <si>
+    <t>091511100174</t>
+  </si>
+  <si>
     <t>CUCHILLA STANDARD S</t>
   </si>
   <si>
     <t>85213</t>
   </si>
   <si>
+    <t>091511100273</t>
+  </si>
+  <si>
     <t>CUCHILLA STANDARD SAC-1</t>
   </si>
   <si>
     <t>85214</t>
   </si>
   <si>
+    <t>091511100280</t>
+  </si>
+  <si>
     <t>CUCHILLA STANDARD SPC-1 (INDIVIDUAL)</t>
   </si>
   <si>
     <t>85216</t>
   </si>
   <si>
+    <t>091511100143</t>
+  </si>
+  <si>
     <t>CUCHILLA STANDARD SVR-1</t>
   </si>
   <si>
@@ -331,66 +460,99 @@
     <t>85886</t>
   </si>
   <si>
+    <t>91511230970</t>
+  </si>
+  <si>
     <t>CUCHILLA WD-AL/BRN</t>
   </si>
   <si>
     <t>85885</t>
   </si>
   <si>
+    <t>91511230963</t>
+  </si>
+  <si>
     <t>CUCHILLA WD-L/BRN</t>
   </si>
   <si>
     <t>85218</t>
   </si>
   <si>
+    <t>091511300703</t>
+  </si>
+  <si>
     <t>PLANCHA CORTE CM-A1 92X61CM (2MM ESPESOR)</t>
   </si>
   <si>
     <t>85220</t>
   </si>
   <si>
+    <t>091511300390</t>
+  </si>
+  <si>
     <t>PLANCHA CORTE CM-A3 43X30 CM (2 MM ESPESOR)</t>
   </si>
   <si>
     <t>85226</t>
   </si>
   <si>
+    <t>91511300512</t>
+  </si>
+  <si>
     <t>PLANCHA CORTE RM-IC-S 60X45 CMS (1.5 MM ESPESOR)</t>
   </si>
   <si>
     <t>85229</t>
   </si>
   <si>
+    <t>091511501216</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA (NEGRO) ASBB-10 X 10</t>
   </si>
   <si>
     <t>85230</t>
   </si>
   <si>
+    <t>091511500332</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA AB-50</t>
   </si>
   <si>
     <t>85700</t>
   </si>
   <si>
+    <t>091511501063</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA AB-SOL-50</t>
   </si>
   <si>
     <t>85231</t>
   </si>
   <si>
+    <t>091511500707</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA ASB-10</t>
   </si>
   <si>
     <t>85234</t>
   </si>
   <si>
+    <t>091511500141</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA COB-1 X 15</t>
   </si>
   <si>
     <t>85235</t>
   </si>
   <si>
+    <t>91511500301</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA HB-5B X 5</t>
   </si>
   <si>
@@ -403,6 +565,9 @@
     <t>85238</t>
   </si>
   <si>
+    <t>091511500134</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA KB X 25</t>
   </si>
   <si>
@@ -415,84 +580,126 @@
     <t>85239</t>
   </si>
   <si>
+    <t>091511500455</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA LB-10 X 10</t>
   </si>
   <si>
     <t>85240</t>
   </si>
   <si>
+    <t>091511500325</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA LB-50 X 50</t>
   </si>
   <si>
     <t>85864</t>
   </si>
   <si>
+    <t>091511500776</t>
+  </si>
+  <si>
     <t>REPUESTO DE CUCHILLA LBB-50X50</t>
   </si>
   <si>
     <t>85849</t>
   </si>
   <si>
+    <t>091511230048</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA LFB-5B (SPEED BLADE)</t>
   </si>
   <si>
     <t>85701</t>
   </si>
   <si>
+    <t>091511501056</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA LSOL-10</t>
   </si>
   <si>
     <t>85243</t>
   </si>
   <si>
+    <t>091511501346</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA MTB-10B</t>
   </si>
   <si>
     <t>85241</t>
   </si>
   <si>
+    <t>091511500769</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA (NEGRO) LBB-10 X 10</t>
   </si>
   <si>
     <t>85244</t>
   </si>
   <si>
+    <t>091511500233</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA PB-450 X 5</t>
   </si>
   <si>
     <t>85245</t>
   </si>
   <si>
+    <t>91511500240</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA PB-800 X 3</t>
   </si>
   <si>
     <t>85247</t>
   </si>
   <si>
+    <t>091511500424</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA RB45-1</t>
   </si>
   <si>
     <t>85248</t>
   </si>
   <si>
+    <t>091511501155</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA RSKB-2 X 5</t>
   </si>
   <si>
     <t>85249</t>
   </si>
   <si>
+    <t>091511900224</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA SKB-10</t>
   </si>
   <si>
     <t>85250</t>
   </si>
   <si>
+    <t>091511700220</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA SKB-2 X 5</t>
   </si>
   <si>
     <t>85779</t>
   </si>
   <si>
+    <t>91511430035</t>
+  </si>
+  <si>
     <t>REPUESTO CUCHILLA SKB-2S/10B</t>
   </si>
   <si>
@@ -505,96 +712,144 @@
     <t>85880</t>
   </si>
   <si>
+    <t>09151150126</t>
+  </si>
+  <si>
     <t>REPUESTO DE CUCHILLA HBB-5B</t>
   </si>
   <si>
     <t>85866</t>
   </si>
   <si>
+    <t>091511500394</t>
+  </si>
+  <si>
     <t>REPUESTO DE CUCHILLA LB 10B</t>
   </si>
   <si>
     <t>85869</t>
   </si>
   <si>
+    <t>091511230390</t>
+  </si>
+  <si>
     <t>REPUESTO DE CUCHILLA SKB-16</t>
   </si>
   <si>
     <t>85822</t>
   </si>
   <si>
+    <t>4051661010675</t>
+  </si>
+  <si>
     <t>ENGRAPADOR ESCRITORIO FM14</t>
   </si>
   <si>
     <t>85288</t>
   </si>
   <si>
+    <t>7313465106020</t>
+  </si>
+  <si>
     <t>ENGRAPADOR ALICATE K1 CLASICA</t>
   </si>
   <si>
     <t>85696</t>
   </si>
   <si>
+    <t>4051661016561</t>
+  </si>
+  <si>
     <t>ENGRAPADOR ALICATE K1 NEGRO</t>
   </si>
   <si>
     <t>85694</t>
   </si>
   <si>
+    <t>4051661016578</t>
+  </si>
+  <si>
     <t>ENGRAPADOR ALICATE K1 BLANCO</t>
   </si>
   <si>
     <t>85695</t>
   </si>
   <si>
+    <t>4051661016585</t>
+  </si>
+  <si>
     <t>ENGRAPADOR ALICATE K1 CELESTE</t>
   </si>
   <si>
     <t>85697</t>
   </si>
   <si>
+    <t>4051661016592</t>
+  </si>
+  <si>
     <t>ENGRAPADOR ALICATE K1 ROSADO</t>
   </si>
   <si>
     <t>85693</t>
   </si>
   <si>
+    <t>4051661016608</t>
+  </si>
+  <si>
     <t>ENGRAPADOR ALICATE K1 VERDE PASTEL</t>
   </si>
   <si>
     <t>85304</t>
   </si>
   <si>
+    <t>7313463057003</t>
+  </si>
+  <si>
     <t>ENGRAPADOR ESCRITORIO K2 (100% METAL)</t>
   </si>
   <si>
     <t>85305</t>
   </si>
   <si>
+    <t>7313468882026</t>
+  </si>
+  <si>
     <t>ENGRAPADOR ESCRITORIO K45 CON SACAGRAPAS</t>
   </si>
   <si>
     <t>85356</t>
   </si>
   <si>
+    <t>7313467105021</t>
+  </si>
+  <si>
     <t>GRAPAS RAPID  26/6 X 5000</t>
   </si>
   <si>
     <t>85380</t>
   </si>
   <si>
+    <t>7313469226014</t>
+  </si>
+  <si>
     <t>PERFORADOR HEAVY DUTY HDC65</t>
   </si>
   <si>
     <t>85821</t>
   </si>
   <si>
+    <t>7313460808158</t>
+  </si>
+  <si>
     <t>ENGRAPADOR HEAVY DUTY HD110</t>
   </si>
   <si>
     <t>85379</t>
   </si>
   <si>
+    <t>7313460006004</t>
+  </si>
+  <si>
     <t>PERFORADOR HEAVY DUTY HDC150 (150 HOJAS)</t>
   </si>
   <si>
@@ -607,6 +862,9 @@
     <t>85384</t>
   </si>
   <si>
+    <t>7313460010001</t>
+  </si>
+  <si>
     <t>REPUESTO PERFORADOR HDC150 (PLACAS X 10)</t>
   </si>
   <si>
@@ -619,72 +877,108 @@
     <t>85401</t>
   </si>
   <si>
+    <t>7313463176001</t>
+  </si>
+  <si>
     <t>ENGRAPADOR CLAVADORA  # M10Y "FUN TO FIX"</t>
   </si>
   <si>
     <t>85395</t>
   </si>
   <si>
+    <t>7313465104507</t>
+  </si>
+  <si>
     <t>ENGRAPADOR CLAVADORA  #  23</t>
   </si>
   <si>
     <t>85397</t>
   </si>
   <si>
+    <t>7313465106501</t>
+  </si>
+  <si>
     <t>ENGRAPADOR CLAVADORA  #  33</t>
   </si>
   <si>
     <t>85881</t>
   </si>
   <si>
+    <t>4051661041488</t>
+  </si>
+  <si>
     <t>ENGRAPADOR CLAVADORA R13 CELESTE</t>
   </si>
   <si>
     <t>85882</t>
   </si>
   <si>
+    <t>4051661041495</t>
+  </si>
+  <si>
     <t>ENGRAPADOR CLAVADORA R13 VERDE</t>
   </si>
   <si>
     <t>85883</t>
   </si>
   <si>
+    <t>4051661041501</t>
+  </si>
+  <si>
     <t>ENGRAPADOR CLAVADORA R13 AMARILLO</t>
   </si>
   <si>
     <t>85884</t>
   </si>
   <si>
+    <t>4051661041518</t>
+  </si>
+  <si>
     <t>ENGRAPADOR CLAVADORA R13 ROSADO</t>
   </si>
   <si>
     <t>85595</t>
   </si>
   <si>
+    <t>7705340001108</t>
+  </si>
+  <si>
     <t>ALFILER WINGO X 50 GR</t>
   </si>
   <si>
     <t>85602</t>
   </si>
   <si>
+    <t>7705340001177</t>
+  </si>
+  <si>
     <t>GRAPAS WINGO  13/06 X 5000</t>
   </si>
   <si>
     <t>85186</t>
   </si>
   <si>
+    <t>091511200119</t>
+  </si>
+  <si>
     <t>CUCHILLA HEAVY DUTY L-3</t>
   </si>
   <si>
     <t>85191</t>
   </si>
   <si>
+    <t>091511200379</t>
+  </si>
+  <si>
     <t>CUCHILLA HEAVY DUTY NOL-1</t>
   </si>
   <si>
     <t>85669</t>
   </si>
   <si>
+    <t>7313465980002</t>
+  </si>
+  <si>
     <t>ENGRAPADOR BRAZO DE 12" E15</t>
   </si>
   <si>
@@ -697,6 +991,9 @@
     <t>85286</t>
   </si>
   <si>
+    <t>7313468125004</t>
+  </si>
+  <si>
     <t>ENGRAPADOR ALICATE ECO 26/6 Y 24/6</t>
   </si>
   <si>
@@ -787,6 +1084,9 @@
     <t>85086</t>
   </si>
   <si>
+    <t>4002432116386</t>
+  </si>
+  <si>
     <t>ENMICADORAS I-LAM TURBO A3 250 MICRONES</t>
   </si>
   <si>
@@ -961,6 +1261,9 @@
     <t>85655</t>
   </si>
   <si>
+    <t>091511400809</t>
+  </si>
+  <si>
     <t>RESERVORIO PARA CUCHILLAS USADAS DC-4</t>
   </si>
   <si>
@@ -979,6 +1282,9 @@
     <t>85810</t>
   </si>
   <si>
+    <t>091511300628</t>
+  </si>
+  <si>
     <t>CUCHILLA ROTATIVA RTY-2/DX</t>
   </si>
   <si>
@@ -991,12 +1297,18 @@
     <t>85867</t>
   </si>
   <si>
+    <t>091511300666</t>
+  </si>
+  <si>
     <t>CUCHILLLA ROTATIVA RTY-4</t>
   </si>
   <si>
     <t>85878</t>
   </si>
   <si>
+    <t>09151140040</t>
+  </si>
+  <si>
     <t>CUCHILLLA XH-AL</t>
   </si>
   <si>
@@ -1033,12 +1345,18 @@
     <t>85225</t>
   </si>
   <si>
+    <t>91511300505</t>
+  </si>
+  <si>
     <t>PLANCHA CORTE RM-IC-M 92X61 CMS (1.5 MM ESPESOR)</t>
   </si>
   <si>
     <t>85799</t>
   </si>
   <si>
+    <t>9151130083</t>
+  </si>
+  <si>
     <t>PLANCHA CORTE RM-30X30 GIRATORIO</t>
   </si>
   <si>
@@ -1093,12 +1411,18 @@
     <t>85573</t>
   </si>
   <si>
+    <t>091511400410</t>
+  </si>
+  <si>
     <t>TIJERA HEAVY DUTY SCS-2 (173 MM)</t>
   </si>
   <si>
     <t>85574</t>
   </si>
   <si>
+    <t>091511100396</t>
+  </si>
+  <si>
     <t>TIJERA STANDARD SCS-3 (160 MM)</t>
   </si>
   <si>
@@ -1183,30 +1507,45 @@
     <t>85872</t>
   </si>
   <si>
+    <t>3221631095198</t>
+  </si>
+  <si>
     <t>GRAPAS RAPID 13/6 X 1600</t>
   </si>
   <si>
     <t>85873</t>
   </si>
   <si>
+    <t>3221631095204</t>
+  </si>
+  <si>
     <t>GRAPAS RAPID 13/8 X 1600</t>
   </si>
   <si>
     <t>85599</t>
   </si>
   <si>
+    <t>7705340001139</t>
+  </si>
+  <si>
     <t>CLIP MARIPOSA # 2 (CAJA X 50)</t>
   </si>
   <si>
     <t>85597</t>
   </si>
   <si>
+    <t>7705340001122</t>
+  </si>
+  <si>
     <t>CLIP JUMBO X 100 WINGO</t>
   </si>
   <si>
     <t>85598</t>
   </si>
   <si>
+    <t>7705340001146</t>
+  </si>
+  <si>
     <t>CLIP MARIPOSA # 1 (CAJA X 12)</t>
   </si>
   <si>
@@ -1217,6 +1556,9 @@
   </si>
   <si>
     <t>85609</t>
+  </si>
+  <si>
+    <t>7705340001030</t>
   </si>
   <si>
     <t>GRAPAS WINGO B-8 X 5000</t>
@@ -1725,10 +2067,10 @@
         <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3">
         <v>80</v>
@@ -1745,13 +2087,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E4">
         <v>80</v>
@@ -1768,13 +2110,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E5">
         <v>50</v>
@@ -1791,13 +2133,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="C6" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E6">
         <v>200</v>
@@ -1814,13 +2156,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E7">
         <v>120</v>
@@ -1837,13 +2179,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="D8" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E8">
         <v>120</v>
@@ -1860,13 +2202,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="E9">
         <v>240</v>
@@ -1883,13 +2225,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E10">
         <v>200</v>
@@ -1906,13 +2248,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="C11" t="s">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="D11" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="E11">
         <v>240</v>
@@ -1921,7 +2263,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1929,13 +2271,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="E12">
         <v>60</v>
@@ -1952,13 +2294,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="E13">
         <v>120</v>
@@ -1975,13 +2317,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="C14" t="s">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="E14">
         <v>120</v>
@@ -1998,13 +2340,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C15" t="s">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="E15">
         <v>120</v>
@@ -2021,13 +2363,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C16" t="s">
-        <v>8</v>
+        <v>51</v>
       </c>
       <c r="D16" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="E16">
         <v>120</v>
@@ -2044,13 +2386,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C17" t="s">
-        <v>8</v>
+        <v>54</v>
       </c>
       <c r="D17" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="E17">
         <v>120</v>
@@ -2067,13 +2409,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C18" t="s">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="D18" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="E18">
         <v>120</v>
@@ -2090,13 +2432,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="C19" t="s">
-        <v>8</v>
+        <v>60</v>
       </c>
       <c r="D19" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="E19">
         <v>120</v>
@@ -2113,13 +2455,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="C20" t="s">
-        <v>8</v>
+        <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>47</v>
+        <v>64</v>
       </c>
       <c r="E20">
         <v>120</v>
@@ -2136,13 +2478,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="C21" t="s">
-        <v>8</v>
+        <v>66</v>
       </c>
       <c r="D21" t="s">
-        <v>49</v>
+        <v>67</v>
       </c>
       <c r="E21">
         <v>120</v>
@@ -2159,13 +2501,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>68</v>
       </c>
       <c r="C22" t="s">
-        <v>8</v>
+        <v>69</v>
       </c>
       <c r="D22" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="E22">
         <v>120</v>
@@ -2182,13 +2524,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
-        <v>8</v>
+        <v>72</v>
       </c>
       <c r="D23" t="s">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="E23">
         <v>60</v>
@@ -2197,7 +2539,7 @@
         <v>3</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -2205,13 +2547,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>8</v>
+        <v>76</v>
       </c>
       <c r="D24" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="E24">
         <v>120</v>
@@ -2228,13 +2570,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="C25" t="s">
-        <v>8</v>
+        <v>79</v>
       </c>
       <c r="D25" t="s">
-        <v>58</v>
+        <v>80</v>
       </c>
       <c r="E25">
         <v>120</v>
@@ -2251,13 +2593,13 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
       <c r="C26" t="s">
-        <v>8</v>
+        <v>82</v>
       </c>
       <c r="D26" t="s">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="E26">
         <v>120</v>
@@ -2274,13 +2616,13 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="C27" t="s">
-        <v>8</v>
+        <v>85</v>
       </c>
       <c r="D27" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="E27">
         <v>120</v>
@@ -2297,13 +2639,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="C28" t="s">
-        <v>8</v>
+        <v>88</v>
       </c>
       <c r="D28" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="E28">
         <v>120</v>
@@ -2320,13 +2662,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="C29" t="s">
-        <v>8</v>
+        <v>91</v>
       </c>
       <c r="D29" t="s">
-        <v>66</v>
+        <v>92</v>
       </c>
       <c r="E29">
         <v>72</v>
@@ -2343,13 +2685,13 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="C30" t="s">
-        <v>8</v>
+        <v>94</v>
       </c>
       <c r="D30" t="s">
-        <v>68</v>
+        <v>95</v>
       </c>
       <c r="E30">
         <v>120</v>
@@ -2366,13 +2708,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>69</v>
+        <v>96</v>
       </c>
       <c r="C31" t="s">
-        <v>8</v>
+        <v>97</v>
       </c>
       <c r="D31" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
       <c r="E31">
         <v>120</v>
@@ -2389,13 +2731,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>71</v>
+        <v>99</v>
       </c>
       <c r="C32" t="s">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="D32" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="E32">
         <v>120</v>
@@ -2412,13 +2754,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>102</v>
       </c>
       <c r="C33" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D33" t="s">
-        <v>74</v>
+        <v>104</v>
       </c>
       <c r="E33">
         <v>144</v>
@@ -2427,7 +2769,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
@@ -2435,13 +2777,13 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>105</v>
       </c>
       <c r="C34" t="s">
-        <v>8</v>
+        <v>106</v>
       </c>
       <c r="D34" t="s">
-        <v>76</v>
+        <v>107</v>
       </c>
       <c r="E34">
         <v>120</v>
@@ -2458,13 +2800,13 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>77</v>
+        <v>108</v>
       </c>
       <c r="C35" t="s">
-        <v>8</v>
+        <v>109</v>
       </c>
       <c r="D35" t="s">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="E35">
         <v>128</v>
@@ -2473,7 +2815,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
@@ -2481,13 +2823,13 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>79</v>
+        <v>111</v>
       </c>
       <c r="C36" t="s">
-        <v>8</v>
+        <v>112</v>
       </c>
       <c r="D36" t="s">
-        <v>80</v>
+        <v>113</v>
       </c>
       <c r="E36">
         <v>120</v>
@@ -2504,13 +2846,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="C37" t="s">
-        <v>8</v>
+        <v>115</v>
       </c>
       <c r="D37" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="E37">
         <v>240</v>
@@ -2527,13 +2869,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>83</v>
+        <v>117</v>
       </c>
       <c r="C38" t="s">
-        <v>8</v>
+        <v>118</v>
       </c>
       <c r="D38" t="s">
-        <v>84</v>
+        <v>119</v>
       </c>
       <c r="E38">
         <v>120</v>
@@ -2550,13 +2892,13 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>85</v>
+        <v>120</v>
       </c>
       <c r="C39" t="s">
-        <v>8</v>
+        <v>121</v>
       </c>
       <c r="D39" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
       <c r="E39">
         <v>240</v>
@@ -2573,13 +2915,13 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>87</v>
+        <v>123</v>
       </c>
       <c r="C40" t="s">
-        <v>8</v>
+        <v>124</v>
       </c>
       <c r="D40" t="s">
-        <v>88</v>
+        <v>125</v>
       </c>
       <c r="E40">
         <v>240</v>
@@ -2596,13 +2938,13 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>89</v>
+        <v>126</v>
       </c>
       <c r="C41" t="s">
-        <v>8</v>
+        <v>127</v>
       </c>
       <c r="D41" t="s">
-        <v>90</v>
+        <v>128</v>
       </c>
       <c r="E41">
         <v>240</v>
@@ -2619,13 +2961,13 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>91</v>
+        <v>129</v>
       </c>
       <c r="C42" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D42" t="s">
-        <v>92</v>
+        <v>130</v>
       </c>
       <c r="E42">
         <v>240</v>
@@ -2642,13 +2984,13 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>93</v>
+        <v>131</v>
       </c>
       <c r="C43" t="s">
-        <v>8</v>
+        <v>132</v>
       </c>
       <c r="D43" t="s">
-        <v>94</v>
+        <v>133</v>
       </c>
       <c r="E43">
         <v>240</v>
@@ -2665,13 +3007,13 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>95</v>
+        <v>134</v>
       </c>
       <c r="C44" t="s">
-        <v>8</v>
+        <v>135</v>
       </c>
       <c r="D44" t="s">
-        <v>96</v>
+        <v>136</v>
       </c>
       <c r="E44">
         <v>480</v>
@@ -2688,13 +3030,13 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>97</v>
+        <v>137</v>
       </c>
       <c r="C45" t="s">
-        <v>8</v>
+        <v>138</v>
       </c>
       <c r="D45" t="s">
-        <v>98</v>
+        <v>139</v>
       </c>
       <c r="E45">
         <v>240</v>
@@ -2711,13 +3053,13 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="C46" t="s">
-        <v>8</v>
+        <v>141</v>
       </c>
       <c r="D46" t="s">
-        <v>100</v>
+        <v>142</v>
       </c>
       <c r="E46">
         <v>800</v>
@@ -2734,13 +3076,13 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>101</v>
+        <v>143</v>
       </c>
       <c r="C47" t="s">
-        <v>8</v>
+        <v>144</v>
       </c>
       <c r="D47" t="s">
-        <v>102</v>
+        <v>145</v>
       </c>
       <c r="E47">
         <v>240</v>
@@ -2757,13 +3099,13 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>103</v>
+        <v>146</v>
       </c>
       <c r="C48" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D48" t="s">
-        <v>104</v>
+        <v>147</v>
       </c>
       <c r="E48">
         <v>120</v>
@@ -2780,13 +3122,13 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>105</v>
+        <v>148</v>
       </c>
       <c r="C49" t="s">
-        <v>8</v>
+        <v>149</v>
       </c>
       <c r="D49" t="s">
-        <v>106</v>
+        <v>150</v>
       </c>
       <c r="E49">
         <v>120</v>
@@ -2803,13 +3145,13 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>107</v>
+        <v>151</v>
       </c>
       <c r="C50" t="s">
-        <v>8</v>
+        <v>152</v>
       </c>
       <c r="D50" t="s">
-        <v>108</v>
+        <v>153</v>
       </c>
       <c r="E50">
         <v>120</v>
@@ -2826,13 +3168,13 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>109</v>
+        <v>154</v>
       </c>
       <c r="C51" t="s">
-        <v>8</v>
+        <v>155</v>
       </c>
       <c r="D51" t="s">
-        <v>110</v>
+        <v>156</v>
       </c>
       <c r="E51">
         <v>10</v>
@@ -2849,13 +3191,13 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>111</v>
+        <v>157</v>
       </c>
       <c r="C52" t="s">
-        <v>8</v>
+        <v>158</v>
       </c>
       <c r="D52" t="s">
-        <v>112</v>
+        <v>159</v>
       </c>
       <c r="E52">
         <v>60</v>
@@ -2872,13 +3214,13 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>113</v>
+        <v>160</v>
       </c>
       <c r="C53" t="s">
-        <v>8</v>
+        <v>161</v>
       </c>
       <c r="D53" t="s">
-        <v>114</v>
+        <v>162</v>
       </c>
       <c r="E53">
         <v>20</v>
@@ -2895,13 +3237,13 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>115</v>
+        <v>163</v>
       </c>
       <c r="C54" t="s">
-        <v>8</v>
+        <v>164</v>
       </c>
       <c r="D54" t="s">
-        <v>116</v>
+        <v>165</v>
       </c>
       <c r="E54">
         <v>720</v>
@@ -2918,13 +3260,13 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>117</v>
+        <v>166</v>
       </c>
       <c r="C55" t="s">
-        <v>8</v>
+        <v>167</v>
       </c>
       <c r="D55" t="s">
-        <v>118</v>
+        <v>168</v>
       </c>
       <c r="E55">
         <v>120</v>
@@ -2941,13 +3283,13 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>119</v>
+        <v>169</v>
       </c>
       <c r="C56" t="s">
-        <v>8</v>
+        <v>170</v>
       </c>
       <c r="D56" t="s">
-        <v>120</v>
+        <v>171</v>
       </c>
       <c r="E56">
         <v>120</v>
@@ -2956,7 +3298,7 @@
         <v>0</v>
       </c>
       <c r="G56" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
@@ -2964,13 +3306,13 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>121</v>
+        <v>172</v>
       </c>
       <c r="C57" t="s">
-        <v>8</v>
+        <v>173</v>
       </c>
       <c r="D57" t="s">
-        <v>122</v>
+        <v>174</v>
       </c>
       <c r="E57">
         <v>720</v>
@@ -2987,13 +3329,13 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>123</v>
+        <v>175</v>
       </c>
       <c r="C58" t="s">
-        <v>8</v>
+        <v>176</v>
       </c>
       <c r="D58" t="s">
-        <v>124</v>
+        <v>177</v>
       </c>
       <c r="E58">
         <v>240</v>
@@ -3010,13 +3352,13 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>125</v>
+        <v>178</v>
       </c>
       <c r="C59" t="s">
-        <v>8</v>
+        <v>179</v>
       </c>
       <c r="D59" t="s">
-        <v>126</v>
+        <v>180</v>
       </c>
       <c r="E59">
         <v>120</v>
@@ -3025,7 +3367,7 @@
         <v>0</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
@@ -3033,13 +3375,13 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>127</v>
+        <v>181</v>
       </c>
       <c r="C60" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D60" t="s">
-        <v>128</v>
+        <v>182</v>
       </c>
       <c r="E60">
         <v>240</v>
@@ -3048,7 +3390,7 @@
         <v>0</v>
       </c>
       <c r="G60" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
@@ -3056,13 +3398,13 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>129</v>
+        <v>183</v>
       </c>
       <c r="C61" t="s">
-        <v>8</v>
+        <v>184</v>
       </c>
       <c r="D61" t="s">
-        <v>130</v>
+        <v>185</v>
       </c>
       <c r="E61">
         <v>240</v>
@@ -3079,13 +3421,13 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>131</v>
+        <v>186</v>
       </c>
       <c r="C62" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D62" t="s">
-        <v>132</v>
+        <v>187</v>
       </c>
       <c r="E62">
         <v>240</v>
@@ -3102,13 +3444,13 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>133</v>
+        <v>188</v>
       </c>
       <c r="C63" t="s">
-        <v>8</v>
+        <v>189</v>
       </c>
       <c r="D63" t="s">
-        <v>134</v>
+        <v>190</v>
       </c>
       <c r="E63">
         <v>240</v>
@@ -3125,13 +3467,13 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>135</v>
+        <v>191</v>
       </c>
       <c r="C64" t="s">
-        <v>8</v>
+        <v>192</v>
       </c>
       <c r="D64" t="s">
-        <v>136</v>
+        <v>193</v>
       </c>
       <c r="E64">
         <v>60</v>
@@ -3148,13 +3490,13 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>137</v>
+        <v>194</v>
       </c>
       <c r="C65" t="s">
-        <v>8</v>
+        <v>195</v>
       </c>
       <c r="D65" t="s">
-        <v>138</v>
+        <v>196</v>
       </c>
       <c r="E65">
         <v>60</v>
@@ -3171,13 +3513,13 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>139</v>
+        <v>197</v>
       </c>
       <c r="C66" t="s">
-        <v>8</v>
+        <v>198</v>
       </c>
       <c r="D66" t="s">
-        <v>140</v>
+        <v>199</v>
       </c>
       <c r="E66">
         <v>120</v>
@@ -3194,13 +3536,13 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>141</v>
+        <v>200</v>
       </c>
       <c r="C67" t="s">
-        <v>8</v>
+        <v>201</v>
       </c>
       <c r="D67" t="s">
-        <v>142</v>
+        <v>202</v>
       </c>
       <c r="E67">
         <v>240</v>
@@ -3209,7 +3551,7 @@
         <v>0</v>
       </c>
       <c r="G67" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
@@ -3217,13 +3559,13 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>143</v>
+        <v>203</v>
       </c>
       <c r="C68" t="s">
-        <v>8</v>
+        <v>204</v>
       </c>
       <c r="D68" t="s">
-        <v>144</v>
+        <v>205</v>
       </c>
       <c r="E68">
         <v>240</v>
@@ -3240,13 +3582,13 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>145</v>
+        <v>206</v>
       </c>
       <c r="C69" t="s">
-        <v>8</v>
+        <v>207</v>
       </c>
       <c r="D69" t="s">
-        <v>146</v>
+        <v>208</v>
       </c>
       <c r="E69">
         <v>240</v>
@@ -3263,13 +3605,13 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>147</v>
+        <v>209</v>
       </c>
       <c r="C70" t="s">
-        <v>8</v>
+        <v>210</v>
       </c>
       <c r="D70" t="s">
-        <v>148</v>
+        <v>211</v>
       </c>
       <c r="E70">
         <v>240</v>
@@ -3286,13 +3628,13 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>149</v>
+        <v>212</v>
       </c>
       <c r="C71" t="s">
-        <v>8</v>
+        <v>213</v>
       </c>
       <c r="D71" t="s">
-        <v>150</v>
+        <v>214</v>
       </c>
       <c r="E71">
         <v>240</v>
@@ -3301,7 +3643,7 @@
         <v>0</v>
       </c>
       <c r="G71" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
@@ -3309,13 +3651,13 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>151</v>
+        <v>215</v>
       </c>
       <c r="C72" t="s">
-        <v>8</v>
+        <v>216</v>
       </c>
       <c r="D72" t="s">
-        <v>152</v>
+        <v>217</v>
       </c>
       <c r="E72">
         <v>480</v>
@@ -3332,13 +3674,13 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>153</v>
+        <v>218</v>
       </c>
       <c r="C73" t="s">
-        <v>8</v>
+        <v>219</v>
       </c>
       <c r="D73" t="s">
-        <v>154</v>
+        <v>220</v>
       </c>
       <c r="E73">
         <v>240</v>
@@ -3355,13 +3697,13 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>155</v>
+        <v>221</v>
       </c>
       <c r="C74" t="s">
-        <v>8</v>
+        <v>222</v>
       </c>
       <c r="D74" t="s">
-        <v>156</v>
+        <v>223</v>
       </c>
       <c r="E74">
         <v>240</v>
@@ -3378,13 +3720,13 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>157</v>
+        <v>224</v>
       </c>
       <c r="C75" t="s">
-        <v>8</v>
+        <v>225</v>
       </c>
       <c r="D75" t="s">
-        <v>158</v>
+        <v>226</v>
       </c>
       <c r="E75">
         <v>240</v>
@@ -3401,13 +3743,13 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>159</v>
+        <v>227</v>
       </c>
       <c r="C76" t="s">
-        <v>8</v>
+        <v>228</v>
       </c>
       <c r="D76" t="s">
-        <v>160</v>
+        <v>229</v>
       </c>
       <c r="E76">
         <v>240</v>
@@ -3416,7 +3758,7 @@
         <v>0</v>
       </c>
       <c r="G76" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
@@ -3424,13 +3766,13 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>161</v>
+        <v>230</v>
       </c>
       <c r="C77" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D77" t="s">
-        <v>162</v>
+        <v>231</v>
       </c>
       <c r="E77">
         <v>600</v>
@@ -3447,13 +3789,13 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>163</v>
+        <v>232</v>
       </c>
       <c r="C78" t="s">
-        <v>8</v>
+        <v>233</v>
       </c>
       <c r="D78" t="s">
-        <v>164</v>
+        <v>234</v>
       </c>
       <c r="E78">
         <v>120</v>
@@ -3470,13 +3812,13 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>165</v>
+        <v>235</v>
       </c>
       <c r="C79" t="s">
-        <v>8</v>
+        <v>236</v>
       </c>
       <c r="D79" t="s">
-        <v>166</v>
+        <v>237</v>
       </c>
       <c r="E79">
         <v>120</v>
@@ -3485,7 +3827,7 @@
         <v>4</v>
       </c>
       <c r="G79" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
@@ -3493,13 +3835,13 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>167</v>
+        <v>238</v>
       </c>
       <c r="C80" t="s">
-        <v>8</v>
+        <v>239</v>
       </c>
       <c r="D80" t="s">
-        <v>168</v>
+        <v>240</v>
       </c>
       <c r="E80">
         <v>60</v>
@@ -3516,13 +3858,13 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>169</v>
+        <v>241</v>
       </c>
       <c r="C81" t="s">
-        <v>8</v>
+        <v>242</v>
       </c>
       <c r="D81" t="s">
-        <v>170</v>
+        <v>243</v>
       </c>
       <c r="E81">
         <v>20</v>
@@ -3539,13 +3881,13 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>171</v>
+        <v>244</v>
       </c>
       <c r="C82" t="s">
-        <v>8</v>
+        <v>245</v>
       </c>
       <c r="D82" t="s">
-        <v>172</v>
+        <v>246</v>
       </c>
       <c r="E82">
         <v>40</v>
@@ -3562,13 +3904,13 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>173</v>
+        <v>247</v>
       </c>
       <c r="C83" t="s">
-        <v>8</v>
+        <v>248</v>
       </c>
       <c r="D83" t="s">
-        <v>174</v>
+        <v>249</v>
       </c>
       <c r="E83">
         <v>40</v>
@@ -3577,7 +3919,7 @@
         <v>0</v>
       </c>
       <c r="G83" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
@@ -3585,13 +3927,13 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>175</v>
+        <v>250</v>
       </c>
       <c r="C84" t="s">
-        <v>8</v>
+        <v>251</v>
       </c>
       <c r="D84" t="s">
-        <v>176</v>
+        <v>252</v>
       </c>
       <c r="E84">
         <v>40</v>
@@ -3608,13 +3950,13 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>177</v>
+        <v>253</v>
       </c>
       <c r="C85" t="s">
-        <v>8</v>
+        <v>254</v>
       </c>
       <c r="D85" t="s">
-        <v>178</v>
+        <v>255</v>
       </c>
       <c r="E85">
         <v>40</v>
@@ -3623,7 +3965,7 @@
         <v>0</v>
       </c>
       <c r="G85" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
@@ -3631,13 +3973,13 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>179</v>
+        <v>256</v>
       </c>
       <c r="C86" t="s">
-        <v>8</v>
+        <v>257</v>
       </c>
       <c r="D86" t="s">
-        <v>180</v>
+        <v>258</v>
       </c>
       <c r="E86">
         <v>40</v>
@@ -3646,7 +3988,7 @@
         <v>0</v>
       </c>
       <c r="G86" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
@@ -3654,13 +3996,13 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>181</v>
+        <v>259</v>
       </c>
       <c r="C87" t="s">
-        <v>8</v>
+        <v>260</v>
       </c>
       <c r="D87" t="s">
-        <v>182</v>
+        <v>261</v>
       </c>
       <c r="E87">
         <v>40</v>
@@ -3669,7 +4011,7 @@
         <v>0</v>
       </c>
       <c r="G87" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
@@ -3677,13 +4019,13 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>183</v>
+        <v>262</v>
       </c>
       <c r="C88" t="s">
-        <v>8</v>
+        <v>263</v>
       </c>
       <c r="D88" t="s">
-        <v>184</v>
+        <v>264</v>
       </c>
       <c r="E88">
         <v>20</v>
@@ -3692,7 +4034,7 @@
         <v>0</v>
       </c>
       <c r="G88" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
@@ -3700,13 +4042,13 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>185</v>
+        <v>265</v>
       </c>
       <c r="C89" t="s">
-        <v>8</v>
+        <v>266</v>
       </c>
       <c r="D89" t="s">
-        <v>186</v>
+        <v>267</v>
       </c>
       <c r="E89">
         <v>20</v>
@@ -3723,13 +4065,13 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>187</v>
+        <v>268</v>
       </c>
       <c r="C90" t="s">
-        <v>8</v>
+        <v>269</v>
       </c>
       <c r="D90" t="s">
-        <v>188</v>
+        <v>270</v>
       </c>
       <c r="E90">
         <v>100</v>
@@ -3746,13 +4088,13 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>189</v>
+        <v>271</v>
       </c>
       <c r="C91" t="s">
-        <v>8</v>
+        <v>272</v>
       </c>
       <c r="D91" t="s">
-        <v>190</v>
+        <v>273</v>
       </c>
       <c r="E91">
         <v>10</v>
@@ -3769,13 +4111,13 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>191</v>
+        <v>274</v>
       </c>
       <c r="C92" t="s">
-        <v>8</v>
+        <v>275</v>
       </c>
       <c r="D92" t="s">
-        <v>192</v>
+        <v>276</v>
       </c>
       <c r="E92">
         <v>10</v>
@@ -3792,13 +4134,13 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>193</v>
+        <v>277</v>
       </c>
       <c r="C93" t="s">
-        <v>8</v>
+        <v>278</v>
       </c>
       <c r="D93" t="s">
-        <v>194</v>
+        <v>279</v>
       </c>
       <c r="E93">
         <v>2</v>
@@ -3815,13 +4157,13 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>195</v>
+        <v>280</v>
       </c>
       <c r="C94" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D94" t="s">
-        <v>196</v>
+        <v>281</v>
       </c>
       <c r="E94">
         <v>6</v>
@@ -3838,13 +4180,13 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>197</v>
+        <v>282</v>
       </c>
       <c r="C95" t="s">
-        <v>8</v>
+        <v>283</v>
       </c>
       <c r="D95" t="s">
-        <v>198</v>
+        <v>284</v>
       </c>
       <c r="E95">
         <v>120</v>
@@ -3853,7 +4195,7 @@
         <v>0</v>
       </c>
       <c r="G95" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
@@ -3861,13 +4203,13 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>199</v>
+        <v>285</v>
       </c>
       <c r="C96" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D96" t="s">
-        <v>200</v>
+        <v>286</v>
       </c>
       <c r="E96">
         <v>120</v>
@@ -3876,7 +4218,7 @@
         <v>0</v>
       </c>
       <c r="G96" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.25">
@@ -3884,13 +4226,13 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>201</v>
+        <v>287</v>
       </c>
       <c r="C97" t="s">
-        <v>8</v>
+        <v>288</v>
       </c>
       <c r="D97" t="s">
-        <v>202</v>
+        <v>289</v>
       </c>
       <c r="E97">
         <v>10</v>
@@ -3899,7 +4241,7 @@
         <v>7</v>
       </c>
       <c r="G97" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.25">
@@ -3907,13 +4249,13 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>203</v>
+        <v>290</v>
       </c>
       <c r="C98" t="s">
-        <v>8</v>
+        <v>291</v>
       </c>
       <c r="D98" t="s">
-        <v>204</v>
+        <v>292</v>
       </c>
       <c r="E98">
         <v>5</v>
@@ -3922,7 +4264,7 @@
         <v>0</v>
       </c>
       <c r="G98" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.25">
@@ -3930,13 +4272,13 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>205</v>
+        <v>293</v>
       </c>
       <c r="C99" t="s">
-        <v>8</v>
+        <v>294</v>
       </c>
       <c r="D99" t="s">
-        <v>206</v>
+        <v>295</v>
       </c>
       <c r="E99">
         <v>5</v>
@@ -3945,7 +4287,7 @@
         <v>0</v>
       </c>
       <c r="G99" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.25">
@@ -3953,13 +4295,13 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>207</v>
+        <v>296</v>
       </c>
       <c r="C100" t="s">
-        <v>8</v>
+        <v>297</v>
       </c>
       <c r="D100" t="s">
-        <v>208</v>
+        <v>298</v>
       </c>
       <c r="E100">
         <v>6</v>
@@ -3976,13 +4318,13 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>209</v>
+        <v>299</v>
       </c>
       <c r="C101" t="s">
-        <v>8</v>
+        <v>300</v>
       </c>
       <c r="D101" t="s">
-        <v>210</v>
+        <v>301</v>
       </c>
       <c r="E101">
         <v>6</v>
@@ -3999,13 +4341,13 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>211</v>
+        <v>302</v>
       </c>
       <c r="C102" t="s">
-        <v>8</v>
+        <v>303</v>
       </c>
       <c r="D102" t="s">
-        <v>212</v>
+        <v>304</v>
       </c>
       <c r="E102">
         <v>6</v>
@@ -4022,13 +4364,13 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>213</v>
+        <v>305</v>
       </c>
       <c r="C103" t="s">
-        <v>8</v>
+        <v>306</v>
       </c>
       <c r="D103" t="s">
-        <v>214</v>
+        <v>307</v>
       </c>
       <c r="E103">
         <v>6</v>
@@ -4045,13 +4387,13 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>215</v>
+        <v>308</v>
       </c>
       <c r="C104" t="s">
-        <v>8</v>
+        <v>309</v>
       </c>
       <c r="D104" t="s">
-        <v>216</v>
+        <v>310</v>
       </c>
       <c r="E104">
         <v>200</v>
@@ -4060,7 +4402,7 @@
         <v>4</v>
       </c>
       <c r="G104" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.25">
@@ -4068,13 +4410,13 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>217</v>
+        <v>311</v>
       </c>
       <c r="C105" t="s">
-        <v>8</v>
+        <v>312</v>
       </c>
       <c r="D105" t="s">
-        <v>218</v>
+        <v>313</v>
       </c>
       <c r="E105">
         <v>56</v>
@@ -4091,13 +4433,13 @@
         <v>105</v>
       </c>
       <c r="B106" t="s">
-        <v>219</v>
+        <v>314</v>
       </c>
       <c r="C106" t="s">
-        <v>8</v>
+        <v>315</v>
       </c>
       <c r="D106" t="s">
-        <v>220</v>
+        <v>316</v>
       </c>
       <c r="E106">
         <v>120</v>
@@ -4114,13 +4456,13 @@
         <v>106</v>
       </c>
       <c r="B107" t="s">
-        <v>221</v>
+        <v>317</v>
       </c>
       <c r="C107" t="s">
-        <v>8</v>
+        <v>318</v>
       </c>
       <c r="D107" t="s">
-        <v>222</v>
+        <v>319</v>
       </c>
       <c r="E107">
         <v>120</v>
@@ -4129,7 +4471,7 @@
         <v>1</v>
       </c>
       <c r="G107" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.25">
@@ -4137,13 +4479,13 @@
         <v>107</v>
       </c>
       <c r="B108" t="s">
-        <v>223</v>
+        <v>320</v>
       </c>
       <c r="C108" t="s">
-        <v>8</v>
+        <v>321</v>
       </c>
       <c r="D108" t="s">
-        <v>224</v>
+        <v>322</v>
       </c>
       <c r="E108">
         <v>18</v>
@@ -4160,13 +4502,13 @@
         <v>108</v>
       </c>
       <c r="B109" t="s">
-        <v>225</v>
+        <v>323</v>
       </c>
       <c r="C109" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D109" t="s">
-        <v>226</v>
+        <v>324</v>
       </c>
       <c r="E109">
         <v>6</v>
@@ -4175,7 +4517,7 @@
         <v>0</v>
       </c>
       <c r="G109" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.25">
@@ -4183,13 +4525,13 @@
         <v>109</v>
       </c>
       <c r="B110" t="s">
-        <v>227</v>
+        <v>325</v>
       </c>
       <c r="C110" t="s">
-        <v>8</v>
+        <v>326</v>
       </c>
       <c r="D110" t="s">
-        <v>228</v>
+        <v>327</v>
       </c>
       <c r="E110">
         <v>54</v>
@@ -4206,13 +4548,13 @@
         <v>110</v>
       </c>
       <c r="B111" t="s">
-        <v>229</v>
+        <v>328</v>
       </c>
       <c r="C111" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D111" t="s">
-        <v>230</v>
+        <v>329</v>
       </c>
       <c r="E111">
         <v>10</v>
@@ -4221,7 +4563,7 @@
         <v>0</v>
       </c>
       <c r="G111" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.25">
@@ -4229,13 +4571,13 @@
         <v>111</v>
       </c>
       <c r="B112" t="s">
-        <v>231</v>
+        <v>330</v>
       </c>
       <c r="C112" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D112" t="s">
-        <v>232</v>
+        <v>331</v>
       </c>
       <c r="E112">
         <v>12</v>
@@ -4244,7 +4586,7 @@
         <v>0</v>
       </c>
       <c r="G112" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
@@ -4252,13 +4594,13 @@
         <v>112</v>
       </c>
       <c r="B113" t="s">
-        <v>233</v>
+        <v>332</v>
       </c>
       <c r="C113" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D113" t="s">
-        <v>234</v>
+        <v>333</v>
       </c>
       <c r="E113">
         <v>12</v>
@@ -4267,7 +4609,7 @@
         <v>0</v>
       </c>
       <c r="G113" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
@@ -4275,13 +4617,13 @@
         <v>113</v>
       </c>
       <c r="B114" t="s">
-        <v>235</v>
+        <v>334</v>
       </c>
       <c r="C114" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D114" t="s">
-        <v>236</v>
+        <v>335</v>
       </c>
       <c r="E114">
         <v>5</v>
@@ -4298,13 +4640,13 @@
         <v>114</v>
       </c>
       <c r="B115" t="s">
-        <v>237</v>
+        <v>336</v>
       </c>
       <c r="C115" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D115" t="s">
-        <v>238</v>
+        <v>337</v>
       </c>
       <c r="E115">
         <v>800</v>
@@ -4321,13 +4663,13 @@
         <v>115</v>
       </c>
       <c r="B116" t="s">
-        <v>239</v>
+        <v>338</v>
       </c>
       <c r="C116" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D116" t="s">
-        <v>240</v>
+        <v>339</v>
       </c>
       <c r="E116">
         <v>5</v>
@@ -4336,7 +4678,7 @@
         <v>0</v>
       </c>
       <c r="G116" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
@@ -4344,13 +4686,13 @@
         <v>116</v>
       </c>
       <c r="B117" t="s">
-        <v>241</v>
+        <v>340</v>
       </c>
       <c r="C117" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D117" t="s">
-        <v>242</v>
+        <v>341</v>
       </c>
       <c r="E117">
         <v>5</v>
@@ -4359,7 +4701,7 @@
         <v>2</v>
       </c>
       <c r="G117" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
@@ -4367,13 +4709,13 @@
         <v>117</v>
       </c>
       <c r="B118" t="s">
-        <v>243</v>
+        <v>342</v>
       </c>
       <c r="C118" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D118" t="s">
-        <v>244</v>
+        <v>343</v>
       </c>
       <c r="E118">
         <v>10</v>
@@ -4390,13 +4732,13 @@
         <v>118</v>
       </c>
       <c r="B119" t="s">
-        <v>245</v>
+        <v>344</v>
       </c>
       <c r="C119" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D119" t="s">
-        <v>246</v>
+        <v>345</v>
       </c>
       <c r="E119">
         <v>10</v>
@@ -4405,7 +4747,7 @@
         <v>6</v>
       </c>
       <c r="G119" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.25">
@@ -4413,13 +4755,13 @@
         <v>119</v>
       </c>
       <c r="B120" t="s">
-        <v>247</v>
+        <v>346</v>
       </c>
       <c r="C120" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D120" t="s">
-        <v>248</v>
+        <v>347</v>
       </c>
       <c r="E120">
         <v>10</v>
@@ -4436,13 +4778,13 @@
         <v>120</v>
       </c>
       <c r="B121" t="s">
-        <v>249</v>
+        <v>348</v>
       </c>
       <c r="C121" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D121" t="s">
-        <v>250</v>
+        <v>349</v>
       </c>
       <c r="E121">
         <v>6</v>
@@ -4451,7 +4793,7 @@
         <v>0</v>
       </c>
       <c r="G121" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.25">
@@ -4459,13 +4801,13 @@
         <v>121</v>
       </c>
       <c r="B122" t="s">
-        <v>251</v>
+        <v>350</v>
       </c>
       <c r="C122" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D122" t="s">
-        <v>252</v>
+        <v>351</v>
       </c>
       <c r="E122">
         <v>6</v>
@@ -4474,7 +4816,7 @@
         <v>0</v>
       </c>
       <c r="G122" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.25">
@@ -4482,13 +4824,13 @@
         <v>122</v>
       </c>
       <c r="B123" t="s">
-        <v>253</v>
+        <v>352</v>
       </c>
       <c r="C123" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D123" t="s">
-        <v>254</v>
+        <v>353</v>
       </c>
       <c r="E123">
         <v>40</v>
@@ -4505,13 +4847,13 @@
         <v>123</v>
       </c>
       <c r="B124" t="s">
-        <v>255</v>
+        <v>354</v>
       </c>
       <c r="C124" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D124" t="s">
-        <v>256</v>
+        <v>355</v>
       </c>
       <c r="E124">
         <v>4</v>
@@ -4528,13 +4870,13 @@
         <v>124</v>
       </c>
       <c r="B125" t="s">
-        <v>257</v>
+        <v>356</v>
       </c>
       <c r="C125" t="s">
-        <v>8</v>
+        <v>357</v>
       </c>
       <c r="D125" t="s">
-        <v>258</v>
+        <v>358</v>
       </c>
       <c r="E125">
         <v>1</v>
@@ -4543,7 +4885,7 @@
         <v>0</v>
       </c>
       <c r="G125" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.25">
@@ -4551,13 +4893,13 @@
         <v>125</v>
       </c>
       <c r="B126" t="s">
-        <v>259</v>
+        <v>359</v>
       </c>
       <c r="C126" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D126" t="s">
-        <v>260</v>
+        <v>360</v>
       </c>
       <c r="E126">
         <v>4</v>
@@ -4574,13 +4916,13 @@
         <v>126</v>
       </c>
       <c r="B127" t="s">
-        <v>261</v>
+        <v>361</v>
       </c>
       <c r="C127" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D127" t="s">
-        <v>262</v>
+        <v>362</v>
       </c>
       <c r="E127">
         <v>4</v>
@@ -4597,13 +4939,13 @@
         <v>127</v>
       </c>
       <c r="B128" t="s">
-        <v>263</v>
+        <v>363</v>
       </c>
       <c r="C128" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D128" t="s">
-        <v>264</v>
+        <v>364</v>
       </c>
       <c r="E128">
         <v>4</v>
@@ -4620,13 +4962,13 @@
         <v>128</v>
       </c>
       <c r="B129" t="s">
-        <v>265</v>
+        <v>365</v>
       </c>
       <c r="C129" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D129" t="s">
-        <v>266</v>
+        <v>366</v>
       </c>
       <c r="E129">
         <v>1</v>
@@ -4635,7 +4977,7 @@
         <v>4</v>
       </c>
       <c r="G129" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.25">
@@ -4643,13 +4985,13 @@
         <v>129</v>
       </c>
       <c r="B130" t="s">
-        <v>267</v>
+        <v>367</v>
       </c>
       <c r="C130" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D130" t="s">
-        <v>268</v>
+        <v>368</v>
       </c>
       <c r="E130">
         <v>60</v>
@@ -4658,7 +5000,7 @@
         <v>3</v>
       </c>
       <c r="G130" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.25">
@@ -4666,13 +5008,13 @@
         <v>130</v>
       </c>
       <c r="B131" t="s">
-        <v>269</v>
+        <v>369</v>
       </c>
       <c r="C131" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D131" t="s">
-        <v>270</v>
+        <v>370</v>
       </c>
       <c r="E131">
         <v>60</v>
@@ -4689,13 +5031,13 @@
         <v>131</v>
       </c>
       <c r="B132" t="s">
-        <v>271</v>
+        <v>371</v>
       </c>
       <c r="C132" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D132" t="s">
-        <v>272</v>
+        <v>372</v>
       </c>
       <c r="E132">
         <v>60</v>
@@ -4712,13 +5054,13 @@
         <v>132</v>
       </c>
       <c r="B133" t="s">
-        <v>273</v>
+        <v>373</v>
       </c>
       <c r="C133" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D133" t="s">
-        <v>274</v>
+        <v>374</v>
       </c>
       <c r="E133">
         <v>60</v>
@@ -4735,13 +5077,13 @@
         <v>133</v>
       </c>
       <c r="B134" t="s">
-        <v>275</v>
+        <v>375</v>
       </c>
       <c r="C134" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D134" t="s">
-        <v>276</v>
+        <v>376</v>
       </c>
       <c r="E134">
         <v>60</v>
@@ -4758,13 +5100,13 @@
         <v>134</v>
       </c>
       <c r="B135" t="s">
-        <v>277</v>
+        <v>377</v>
       </c>
       <c r="C135" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D135" t="s">
-        <v>278</v>
+        <v>378</v>
       </c>
       <c r="E135">
         <v>60</v>
@@ -4781,13 +5123,13 @@
         <v>135</v>
       </c>
       <c r="B136" t="s">
-        <v>279</v>
+        <v>379</v>
       </c>
       <c r="C136" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D136" t="s">
-        <v>280</v>
+        <v>380</v>
       </c>
       <c r="E136">
         <v>60</v>
@@ -4804,13 +5146,13 @@
         <v>136</v>
       </c>
       <c r="B137" t="s">
-        <v>281</v>
+        <v>381</v>
       </c>
       <c r="C137" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D137" t="s">
-        <v>282</v>
+        <v>382</v>
       </c>
       <c r="E137">
         <v>30</v>
@@ -4827,13 +5169,13 @@
         <v>137</v>
       </c>
       <c r="B138" t="s">
-        <v>283</v>
+        <v>383</v>
       </c>
       <c r="C138" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D138" t="s">
-        <v>284</v>
+        <v>384</v>
       </c>
       <c r="E138">
         <v>40</v>
@@ -4850,13 +5192,13 @@
         <v>138</v>
       </c>
       <c r="B139" t="s">
-        <v>285</v>
+        <v>385</v>
       </c>
       <c r="C139" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D139" t="s">
-        <v>286</v>
+        <v>386</v>
       </c>
       <c r="E139">
         <v>63</v>
@@ -4873,13 +5215,13 @@
         <v>139</v>
       </c>
       <c r="B140" t="s">
-        <v>287</v>
+        <v>387</v>
       </c>
       <c r="C140" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D140" t="s">
-        <v>288</v>
+        <v>388</v>
       </c>
       <c r="E140">
         <v>10</v>
@@ -4896,13 +5238,13 @@
         <v>140</v>
       </c>
       <c r="B141" t="s">
-        <v>289</v>
+        <v>389</v>
       </c>
       <c r="C141" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D141" t="s">
-        <v>290</v>
+        <v>390</v>
       </c>
       <c r="E141">
         <v>40</v>
@@ -4919,13 +5261,13 @@
         <v>141</v>
       </c>
       <c r="B142" t="s">
-        <v>291</v>
+        <v>391</v>
       </c>
       <c r="C142" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D142" t="s">
-        <v>292</v>
+        <v>392</v>
       </c>
       <c r="E142">
         <v>60</v>
@@ -4942,13 +5284,13 @@
         <v>142</v>
       </c>
       <c r="B143" t="s">
-        <v>293</v>
+        <v>393</v>
       </c>
       <c r="C143" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D143" t="s">
-        <v>294</v>
+        <v>394</v>
       </c>
       <c r="E143">
         <v>6</v>
@@ -4965,13 +5307,13 @@
         <v>143</v>
       </c>
       <c r="B144" t="s">
-        <v>295</v>
+        <v>395</v>
       </c>
       <c r="C144" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D144" t="s">
-        <v>296</v>
+        <v>396</v>
       </c>
       <c r="E144">
         <v>18</v>
@@ -4980,7 +5322,7 @@
         <v>0</v>
       </c>
       <c r="G144" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.25">
@@ -4988,13 +5330,13 @@
         <v>144</v>
       </c>
       <c r="B145" t="s">
-        <v>297</v>
+        <v>397</v>
       </c>
       <c r="C145" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D145" t="s">
-        <v>298</v>
+        <v>398</v>
       </c>
       <c r="E145">
         <v>8</v>
@@ -5011,13 +5353,13 @@
         <v>145</v>
       </c>
       <c r="B146" t="s">
-        <v>299</v>
+        <v>399</v>
       </c>
       <c r="C146" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D146" t="s">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="E146">
         <v>30</v>
@@ -5034,13 +5376,13 @@
         <v>146</v>
       </c>
       <c r="B147" t="s">
-        <v>301</v>
+        <v>401</v>
       </c>
       <c r="C147" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D147" t="s">
-        <v>302</v>
+        <v>402</v>
       </c>
       <c r="E147">
         <v>2</v>
@@ -5049,7 +5391,7 @@
         <v>0</v>
       </c>
       <c r="G147" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.25">
@@ -5057,13 +5399,13 @@
         <v>147</v>
       </c>
       <c r="B148" t="s">
-        <v>303</v>
+        <v>403</v>
       </c>
       <c r="C148" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D148" t="s">
-        <v>304</v>
+        <v>404</v>
       </c>
       <c r="E148">
         <v>5</v>
@@ -5080,13 +5422,13 @@
         <v>148</v>
       </c>
       <c r="B149" t="s">
-        <v>305</v>
+        <v>405</v>
       </c>
       <c r="C149" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D149" t="s">
-        <v>306</v>
+        <v>406</v>
       </c>
       <c r="E149">
         <v>5</v>
@@ -5103,13 +5445,13 @@
         <v>149</v>
       </c>
       <c r="B150" t="s">
-        <v>307</v>
+        <v>407</v>
       </c>
       <c r="C150" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D150" t="s">
-        <v>308</v>
+        <v>408</v>
       </c>
       <c r="E150">
         <v>5</v>
@@ -5126,13 +5468,13 @@
         <v>150</v>
       </c>
       <c r="B151" t="s">
-        <v>309</v>
+        <v>409</v>
       </c>
       <c r="C151" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D151" t="s">
-        <v>310</v>
+        <v>410</v>
       </c>
       <c r="E151">
         <v>5</v>
@@ -5149,13 +5491,13 @@
         <v>151</v>
       </c>
       <c r="B152" t="s">
-        <v>311</v>
+        <v>411</v>
       </c>
       <c r="C152" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D152" t="s">
-        <v>312</v>
+        <v>412</v>
       </c>
       <c r="E152">
         <v>20</v>
@@ -5164,7 +5506,7 @@
         <v>8</v>
       </c>
       <c r="G152" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.25">
@@ -5172,13 +5514,13 @@
         <v>152</v>
       </c>
       <c r="B153" t="s">
-        <v>313</v>
+        <v>413</v>
       </c>
       <c r="C153" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D153" t="s">
-        <v>314</v>
+        <v>414</v>
       </c>
       <c r="E153">
         <v>240</v>
@@ -5195,13 +5537,13 @@
         <v>153</v>
       </c>
       <c r="B154" t="s">
-        <v>315</v>
+        <v>415</v>
       </c>
       <c r="C154" t="s">
-        <v>8</v>
+        <v>416</v>
       </c>
       <c r="D154" t="s">
-        <v>316</v>
+        <v>417</v>
       </c>
       <c r="E154">
         <v>120</v>
@@ -5218,13 +5560,13 @@
         <v>154</v>
       </c>
       <c r="B155" t="s">
-        <v>317</v>
+        <v>418</v>
       </c>
       <c r="C155" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D155" t="s">
-        <v>318</v>
+        <v>419</v>
       </c>
       <c r="E155">
         <v>60</v>
@@ -5241,13 +5583,13 @@
         <v>155</v>
       </c>
       <c r="B156" t="s">
-        <v>319</v>
+        <v>420</v>
       </c>
       <c r="C156" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D156" t="s">
-        <v>320</v>
+        <v>421</v>
       </c>
       <c r="E156">
         <v>120</v>
@@ -5256,7 +5598,7 @@
         <v>0</v>
       </c>
       <c r="G156" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.25">
@@ -5264,13 +5606,13 @@
         <v>156</v>
       </c>
       <c r="B157" t="s">
-        <v>321</v>
+        <v>422</v>
       </c>
       <c r="C157" t="s">
-        <v>8</v>
+        <v>423</v>
       </c>
       <c r="D157" t="s">
-        <v>322</v>
+        <v>424</v>
       </c>
       <c r="E157">
         <v>72</v>
@@ -5287,13 +5629,13 @@
         <v>157</v>
       </c>
       <c r="B158" t="s">
-        <v>323</v>
+        <v>425</v>
       </c>
       <c r="C158" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D158" t="s">
-        <v>324</v>
+        <v>426</v>
       </c>
       <c r="E158">
         <v>60</v>
@@ -5310,13 +5652,13 @@
         <v>158</v>
       </c>
       <c r="B159" t="s">
-        <v>325</v>
+        <v>427</v>
       </c>
       <c r="C159" t="s">
-        <v>8</v>
+        <v>428</v>
       </c>
       <c r="D159" t="s">
-        <v>326</v>
+        <v>429</v>
       </c>
       <c r="E159">
         <v>120</v>
@@ -5333,13 +5675,13 @@
         <v>159</v>
       </c>
       <c r="B160" t="s">
-        <v>327</v>
+        <v>430</v>
       </c>
       <c r="C160" t="s">
-        <v>8</v>
+        <v>431</v>
       </c>
       <c r="D160" t="s">
-        <v>328</v>
+        <v>432</v>
       </c>
       <c r="E160">
         <v>72</v>
@@ -5356,13 +5698,13 @@
         <v>160</v>
       </c>
       <c r="B161" t="s">
-        <v>329</v>
+        <v>433</v>
       </c>
       <c r="C161" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D161" t="s">
-        <v>330</v>
+        <v>434</v>
       </c>
       <c r="E161">
         <v>20</v>
@@ -5379,13 +5721,13 @@
         <v>161</v>
       </c>
       <c r="B162" t="s">
-        <v>331</v>
+        <v>435</v>
       </c>
       <c r="C162" t="s">
-        <v>8</v>
+        <v>127</v>
       </c>
       <c r="D162" t="s">
-        <v>332</v>
+        <v>436</v>
       </c>
       <c r="E162">
         <v>100</v>
@@ -5402,13 +5744,13 @@
         <v>162</v>
       </c>
       <c r="B163" t="s">
-        <v>333</v>
+        <v>437</v>
       </c>
       <c r="C163" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D163" t="s">
-        <v>334</v>
+        <v>438</v>
       </c>
       <c r="E163">
         <v>5</v>
@@ -5425,13 +5767,13 @@
         <v>163</v>
       </c>
       <c r="B164" t="s">
-        <v>335</v>
+        <v>439</v>
       </c>
       <c r="C164" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D164" t="s">
-        <v>336</v>
+        <v>440</v>
       </c>
       <c r="E164">
         <v>10</v>
@@ -5440,7 +5782,7 @@
         <v>4</v>
       </c>
       <c r="G164" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.25">
@@ -5448,13 +5790,13 @@
         <v>164</v>
       </c>
       <c r="B165" t="s">
-        <v>337</v>
+        <v>441</v>
       </c>
       <c r="C165" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D165" t="s">
-        <v>338</v>
+        <v>442</v>
       </c>
       <c r="E165">
         <v>20</v>
@@ -5471,13 +5813,13 @@
         <v>165</v>
       </c>
       <c r="B166" t="s">
-        <v>339</v>
+        <v>443</v>
       </c>
       <c r="C166" t="s">
-        <v>8</v>
+        <v>444</v>
       </c>
       <c r="D166" t="s">
-        <v>340</v>
+        <v>445</v>
       </c>
       <c r="E166">
         <v>20</v>
@@ -5494,13 +5836,13 @@
         <v>166</v>
       </c>
       <c r="B167" t="s">
-        <v>341</v>
+        <v>446</v>
       </c>
       <c r="C167" t="s">
-        <v>8</v>
+        <v>447</v>
       </c>
       <c r="D167" t="s">
-        <v>342</v>
+        <v>448</v>
       </c>
       <c r="E167">
         <v>24</v>
@@ -5517,13 +5859,13 @@
         <v>167</v>
       </c>
       <c r="B168" t="s">
-        <v>343</v>
+        <v>449</v>
       </c>
       <c r="C168" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D168" t="s">
-        <v>344</v>
+        <v>450</v>
       </c>
       <c r="E168">
         <v>240</v>
@@ -5540,13 +5882,13 @@
         <v>168</v>
       </c>
       <c r="B169" t="s">
-        <v>345</v>
+        <v>451</v>
       </c>
       <c r="C169" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D169" t="s">
-        <v>346</v>
+        <v>452</v>
       </c>
       <c r="E169">
         <v>240</v>
@@ -5563,13 +5905,13 @@
         <v>169</v>
       </c>
       <c r="B170" t="s">
-        <v>347</v>
+        <v>453</v>
       </c>
       <c r="C170" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D170" t="s">
-        <v>348</v>
+        <v>454</v>
       </c>
       <c r="E170">
         <v>480</v>
@@ -5586,13 +5928,13 @@
         <v>170</v>
       </c>
       <c r="B171" t="s">
-        <v>349</v>
+        <v>455</v>
       </c>
       <c r="C171" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D171" t="s">
-        <v>350</v>
+        <v>456</v>
       </c>
       <c r="E171">
         <v>120</v>
@@ -5609,13 +5951,13 @@
         <v>171</v>
       </c>
       <c r="B172" t="s">
-        <v>351</v>
+        <v>457</v>
       </c>
       <c r="C172" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D172" t="s">
-        <v>352</v>
+        <v>458</v>
       </c>
       <c r="E172">
         <v>240</v>
@@ -5632,13 +5974,13 @@
         <v>172</v>
       </c>
       <c r="B173" t="s">
-        <v>353</v>
+        <v>459</v>
       </c>
       <c r="C173" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D173" t="s">
-        <v>354</v>
+        <v>460</v>
       </c>
       <c r="E173">
         <v>240</v>
@@ -5655,13 +5997,13 @@
         <v>173</v>
       </c>
       <c r="B174" t="s">
-        <v>355</v>
+        <v>461</v>
       </c>
       <c r="C174" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D174" t="s">
-        <v>356</v>
+        <v>462</v>
       </c>
       <c r="E174">
         <v>480</v>
@@ -5678,13 +6020,13 @@
         <v>174</v>
       </c>
       <c r="B175" t="s">
-        <v>357</v>
+        <v>463</v>
       </c>
       <c r="C175" t="s">
-        <v>8</v>
+        <v>431</v>
       </c>
       <c r="D175" t="s">
-        <v>358</v>
+        <v>464</v>
       </c>
       <c r="E175">
         <v>120</v>
@@ -5701,13 +6043,13 @@
         <v>175</v>
       </c>
       <c r="B176" t="s">
-        <v>359</v>
+        <v>465</v>
       </c>
       <c r="C176" t="s">
-        <v>8</v>
+        <v>466</v>
       </c>
       <c r="D176" t="s">
-        <v>360</v>
+        <v>467</v>
       </c>
       <c r="E176">
         <v>120</v>
@@ -5724,13 +6066,13 @@
         <v>176</v>
       </c>
       <c r="B177" t="s">
-        <v>361</v>
+        <v>468</v>
       </c>
       <c r="C177" t="s">
-        <v>8</v>
+        <v>469</v>
       </c>
       <c r="D177" t="s">
-        <v>362</v>
+        <v>470</v>
       </c>
       <c r="E177">
         <v>120</v>
@@ -5747,13 +6089,13 @@
         <v>177</v>
       </c>
       <c r="B178" t="s">
-        <v>363</v>
+        <v>471</v>
       </c>
       <c r="C178" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D178" t="s">
-        <v>364</v>
+        <v>472</v>
       </c>
       <c r="E178">
         <v>12</v>
@@ -5770,13 +6112,13 @@
         <v>178</v>
       </c>
       <c r="B179" t="s">
-        <v>365</v>
+        <v>473</v>
       </c>
       <c r="C179" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D179" t="s">
-        <v>366</v>
+        <v>474</v>
       </c>
       <c r="E179">
         <v>12</v>
@@ -5793,13 +6135,13 @@
         <v>179</v>
       </c>
       <c r="B180" t="s">
-        <v>367</v>
+        <v>475</v>
       </c>
       <c r="C180" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D180" t="s">
-        <v>368</v>
+        <v>476</v>
       </c>
       <c r="E180">
         <v>30</v>
@@ -5808,7 +6150,7 @@
         <v>0</v>
       </c>
       <c r="G180" s="5" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
     </row>
     <row r="181" spans="1:7" x14ac:dyDescent="0.25">
@@ -5816,13 +6158,13 @@
         <v>180</v>
       </c>
       <c r="B181" t="s">
-        <v>369</v>
+        <v>477</v>
       </c>
       <c r="C181" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D181" t="s">
-        <v>370</v>
+        <v>478</v>
       </c>
       <c r="E181">
         <v>12</v>
@@ -5831,7 +6173,7 @@
         <v>4</v>
       </c>
       <c r="G181" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="182" spans="1:7" x14ac:dyDescent="0.25">
@@ -5839,13 +6181,13 @@
         <v>181</v>
       </c>
       <c r="B182" t="s">
-        <v>371</v>
+        <v>479</v>
       </c>
       <c r="C182" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D182" t="s">
-        <v>372</v>
+        <v>480</v>
       </c>
       <c r="E182">
         <v>6</v>
@@ -5854,7 +6196,7 @@
         <v>6</v>
       </c>
       <c r="G182" s="7" t="s">
-        <v>54</v>
+        <v>74</v>
       </c>
     </row>
     <row r="183" spans="1:7" x14ac:dyDescent="0.25">
@@ -5862,13 +6204,13 @@
         <v>182</v>
       </c>
       <c r="B183" t="s">
-        <v>373</v>
+        <v>481</v>
       </c>
       <c r="C183" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D183" t="s">
-        <v>374</v>
+        <v>482</v>
       </c>
       <c r="E183">
         <v>1</v>
@@ -5885,13 +6227,13 @@
         <v>183</v>
       </c>
       <c r="B184" t="s">
-        <v>375</v>
+        <v>483</v>
       </c>
       <c r="C184" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D184" t="s">
-        <v>376</v>
+        <v>484</v>
       </c>
       <c r="E184">
         <v>20</v>
@@ -5908,13 +6250,13 @@
         <v>184</v>
       </c>
       <c r="B185" t="s">
-        <v>377</v>
+        <v>485</v>
       </c>
       <c r="C185" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D185" t="s">
-        <v>378</v>
+        <v>486</v>
       </c>
       <c r="E185">
         <v>20</v>
@@ -5931,13 +6273,13 @@
         <v>185</v>
       </c>
       <c r="B186" t="s">
-        <v>379</v>
+        <v>487</v>
       </c>
       <c r="C186" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D186" t="s">
-        <v>380</v>
+        <v>488</v>
       </c>
       <c r="E186">
         <v>20</v>
@@ -5954,13 +6296,13 @@
         <v>186</v>
       </c>
       <c r="B187" t="s">
-        <v>381</v>
+        <v>489</v>
       </c>
       <c r="C187" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D187" t="s">
-        <v>382</v>
+        <v>490</v>
       </c>
       <c r="E187">
         <v>56</v>
@@ -5977,13 +6319,13 @@
         <v>187</v>
       </c>
       <c r="B188" t="s">
-        <v>383</v>
+        <v>491</v>
       </c>
       <c r="C188" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D188" t="s">
-        <v>384</v>
+        <v>492</v>
       </c>
       <c r="E188">
         <v>50</v>
@@ -6000,13 +6342,13 @@
         <v>188</v>
       </c>
       <c r="B189" t="s">
-        <v>385</v>
+        <v>493</v>
       </c>
       <c r="C189" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D189" t="s">
-        <v>386</v>
+        <v>494</v>
       </c>
       <c r="E189">
         <v>50</v>
@@ -6023,13 +6365,13 @@
         <v>189</v>
       </c>
       <c r="B190" t="s">
-        <v>387</v>
+        <v>495</v>
       </c>
       <c r="C190" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D190" t="s">
-        <v>388</v>
+        <v>496</v>
       </c>
       <c r="E190">
         <v>50</v>
@@ -6046,13 +6388,13 @@
         <v>190</v>
       </c>
       <c r="B191" t="s">
-        <v>389</v>
+        <v>497</v>
       </c>
       <c r="C191" t="s">
-        <v>8</v>
+        <v>498</v>
       </c>
       <c r="D191" t="s">
-        <v>390</v>
+        <v>499</v>
       </c>
       <c r="E191">
         <v>50</v>
@@ -6069,13 +6411,13 @@
         <v>191</v>
       </c>
       <c r="B192" t="s">
-        <v>391</v>
+        <v>500</v>
       </c>
       <c r="C192" t="s">
-        <v>8</v>
+        <v>501</v>
       </c>
       <c r="D192" t="s">
-        <v>392</v>
+        <v>502</v>
       </c>
       <c r="E192">
         <v>50</v>
@@ -6092,13 +6434,13 @@
         <v>192</v>
       </c>
       <c r="B193" t="s">
-        <v>393</v>
+        <v>503</v>
       </c>
       <c r="C193" t="s">
-        <v>8</v>
+        <v>504</v>
       </c>
       <c r="D193" t="s">
-        <v>394</v>
+        <v>505</v>
       </c>
       <c r="E193">
         <v>50</v>
@@ -6115,13 +6457,13 @@
         <v>193</v>
       </c>
       <c r="B194" t="s">
-        <v>395</v>
+        <v>506</v>
       </c>
       <c r="C194" t="s">
-        <v>8</v>
+        <v>507</v>
       </c>
       <c r="D194" t="s">
-        <v>396</v>
+        <v>508</v>
       </c>
       <c r="E194">
         <v>100</v>
@@ -6138,13 +6480,13 @@
         <v>194</v>
       </c>
       <c r="B195" t="s">
-        <v>397</v>
+        <v>509</v>
       </c>
       <c r="C195" t="s">
-        <v>8</v>
+        <v>510</v>
       </c>
       <c r="D195" t="s">
-        <v>398</v>
+        <v>511</v>
       </c>
       <c r="E195">
         <v>60</v>
@@ -6161,13 +6503,13 @@
         <v>195</v>
       </c>
       <c r="B196" t="s">
-        <v>399</v>
+        <v>512</v>
       </c>
       <c r="C196" t="s">
-        <v>8</v>
+        <v>103</v>
       </c>
       <c r="D196" t="s">
-        <v>400</v>
+        <v>513</v>
       </c>
       <c r="E196">
         <v>100</v>
@@ -6184,13 +6526,13 @@
         <v>196</v>
       </c>
       <c r="B197" t="s">
-        <v>401</v>
+        <v>514</v>
       </c>
       <c r="C197" t="s">
-        <v>8</v>
+        <v>515</v>
       </c>
       <c r="D197" t="s">
-        <v>402</v>
+        <v>516</v>
       </c>
       <c r="E197">
         <v>80</v>

</xml_diff>